<commit_message>
Update AR invoice Template final.xlsx
</commit_message>
<xml_diff>
--- a/AR/AR invoice Template final.xlsx
+++ b/AR/AR invoice Template final.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\MSIG BY ALEX\AR\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\MSIGSX\AR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EAE330E0-7235-4FC3-8239-E572A9632DBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA7B5F39-F9F3-4D69-A53A-8DD5071B4BD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="48" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{D3F70513-4056-4EC3-ADC2-9276ACB3237B}"/>
   </bookViews>
@@ -432,7 +432,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2195" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2195" uniqueCount="244">
   <si>
     <t>ParentKey</t>
   </si>
@@ -1161,6 +1161,9 @@
   </si>
   <si>
     <t>200000</t>
+  </si>
+  <si>
+    <t>ON00</t>
   </si>
 </sst>
 </file>
@@ -10683,7 +10686,7 @@
         <v>17</v>
       </c>
       <c r="G21" s="43" t="s">
-        <v>218</v>
+        <v>243</v>
       </c>
       <c r="H21" s="42" t="s">
         <v>18</v>

</xml_diff>